<commit_message>
Update: Threat Alert Report - 2026-03-15 03:16
</commit_message>
<xml_diff>
--- a/excel_routes/route_DMM_ATZ_threats.xlsx
+++ b/excel_routes/route_DMM_ATZ_threats.xlsx
@@ -33,7 +33,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="003498DB"/>
         <bgColor rgb="003498DB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+        <bgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
     <fill>
@@ -71,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -80,6 +92,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -447,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -459,7 +477,7 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -523,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>06-MAR-26</t>
+          <t>16-MAR-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -533,17 +551,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-234</t>
+          <t>Nesma Airlines NE-153</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1023</v>
+        <v>1249</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1226</v>
+        <v>1976</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-203</v>
+        <v>-727</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>30</v>
@@ -556,7 +574,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>HIGH THREAT ALERT - NEED ACTION</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -568,7 +586,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>09-MAR-26</t>
+          <t>16-MAR-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -578,17 +596,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-132</t>
+          <t>Nile Air NP-134</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>914</v>
+        <v>1419</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1226</v>
+        <v>1976</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-312</v>
+        <v>-557</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>30</v>
@@ -599,12 +617,57 @@
       <c r="I3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>20-MAR-26</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SM-438</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Nesma Airlines NE-151</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1249</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1556</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>-307</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>LOW THREAT</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>

</xml_diff>